<commit_message>
feat(medição,chamados,catálogo): BM v2, PDF período estilo BM, histórico operacional e alterações de BD
Unifica e evolui o Boletim de Medição (modelo v2 / GIP, capa e exportação XLSX alinhadas ao padrão institucional) e melhora o fluxo operacional dos chamados: exclusão lógica com filtros/URLs, histórico/timeline e apoio geográfico, materiais no detalhe do operador, e auditoria de quem lançou itens (criado_por). Refatora o PDF «Chamados e anexos» (Dompdf) com identidade BM — capa em faixa roxa, KPIs em cards, cards por chamado, mosaico de fotos e rodapé institucional com paginação. Acrescenta saldo de estoque nos itens do cliente, ajustes de UI/CSS em tabelas e catálogo, modelo/regeneração de templates XLSX, novas migrações (043–045) e atualização do schema.sql; smoke do PDF actualizado.
</commit_message>
<xml_diff>
--- a/assets/templates/boletim_medicao_modelo_1.xlsx
+++ b/assets/templates/boletim_medicao_modelo_1.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="26">
   <si>
     <t>BOLETIM DE MEDIÇÃO  ·  Nº 202605</t>
   </si>
@@ -36,10 +36,10 @@
   <si>
     <t>Período / emitido
 Modelo de referência
-13/05/2026 13:25</t>
-  </si>
-  <si>
-    <t>Manutenção da iluminação pública — medição  ·  LightOn</t>
+15/05/2026 19:57</t>
+  </si>
+  <si>
+    <t>Manutenção da iluminação pública — medição  ·  OnLight</t>
   </si>
   <si>
     <t>DATA</t>
@@ -93,19 +93,13 @@
     <t>Material Retirados/Incluído</t>
   </si>
   <si>
-    <t>Quantidade</t>
-  </si>
-  <si>
-    <t>Marca Luminária</t>
-  </si>
-  <si>
     <t>Nenhum lançamento «utilizado» no período (filtro pela data em chamado_itens.criado_em; defina período nos filtros da lista de chamados).</t>
   </si>
   <si>
     <t>TOTAIS</t>
   </si>
   <si>
-    <t>Documento gerado pelo sistema LightOn · Boletim de medição (modelo GIP) · Gerado por: Sistema</t>
+    <t>Documento gerado pelo sistema OnLight · Boletim de medição (modelo GIP) · Gerado por: Sistema</t>
   </si>
 </sst>
 </file>
@@ -163,7 +157,7 @@
       <name val="Aptos"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -172,8 +166,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1A1A2E"/>
-        <bgColor rgb="FF1A1A2E"/>
+        <fgColor rgb="FF534AB7"/>
+        <bgColor rgb="FF534AB7"/>
       </patternFill>
     </fill>
     <fill>
@@ -186,12 +180,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF534AB7"/>
-        <bgColor rgb="FF534AB7"/>
       </patternFill>
     </fill>
   </fills>
@@ -328,7 +316,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="5" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="2" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
@@ -649,7 +637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="true" style="0"/>
@@ -668,12 +656,10 @@
     <col min="14" max="14" width="8" customWidth="true" style="0"/>
     <col min="15" max="15" width="18" customWidth="true" style="0"/>
     <col min="16" max="16" width="18" customWidth="true" style="0"/>
-    <col min="17" max="17" width="24" customWidth="true" style="0"/>
-    <col min="18" max="18" width="12" customWidth="true" style="0"/>
-    <col min="19" max="19" width="22" customWidth="true" style="0"/>
+    <col min="17" max="17" width="28" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" customHeight="1" ht="54">
+    <row r="1" spans="1:17" customHeight="1" ht="54">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -693,10 +679,8 @@
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
     </row>
-    <row r="2" spans="1:19" customHeight="1" ht="24">
+    <row r="2" spans="1:17" customHeight="1" ht="24">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -721,11 +705,9 @@
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
-      <c r="S2" s="5"/>
+      <c r="Q2" s="5"/>
     </row>
-    <row r="3" spans="1:19" customHeight="1" ht="36">
+    <row r="3" spans="1:17" customHeight="1" ht="36">
       <c r="A3" s="6" t="s">
         <v>5</v>
       </c>
@@ -745,10 +727,8 @@
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
       <c r="Q3" s="6"/>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6"/>
     </row>
-    <row r="4" spans="1:19" customHeight="1" ht="8">
+    <row r="4" spans="1:17" customHeight="1" ht="8">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -766,10 +746,8 @@
       <c r="O4" s="7"/>
       <c r="P4" s="7"/>
       <c r="Q4" s="7"/>
-      <c r="R4" s="7"/>
-      <c r="S4" s="7"/>
     </row>
-    <row r="5" spans="1:19" customHeight="1" ht="40">
+    <row r="5" spans="1:17" customHeight="1" ht="40">
       <c r="A5" s="8" t="s">
         <v>6</v>
       </c>
@@ -821,16 +799,10 @@
       <c r="Q5" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="R5" s="8" t="s">
+    </row>
+    <row r="6" spans="1:17">
+      <c r="A6" s="9" t="s">
         <v>23</v>
-      </c>
-      <c r="S5" s="8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19">
-      <c r="A6" s="9" t="s">
-        <v>25</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -848,12 +820,10 @@
       <c r="O6" s="9"/>
       <c r="P6" s="9"/>
       <c r="Q6" s="9"/>
-      <c r="R6" s="9"/>
-      <c r="S6" s="9"/>
     </row>
-    <row r="7" spans="1:19">
+    <row r="7" spans="1:17">
       <c r="A7" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -875,12 +845,10 @@
         <v>0.0</v>
       </c>
       <c r="Q7" s="11"/>
-      <c r="R7" s="11"/>
-      <c r="S7" s="11"/>
     </row>
-    <row r="8" spans="1:19">
+    <row r="8" spans="1:17">
       <c r="A8" s="14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B8" s="14"/>
       <c r="C8" s="14"/>
@@ -898,27 +866,25 @@
       <c r="O8" s="14"/>
       <c r="P8" s="14"/>
       <c r="Q8" s="14"/>
-      <c r="R8" s="14"/>
-      <c r="S8" s="14"/>
     </row>
   </sheetData>
   <mergeCells>
-    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="E2:H2"/>
     <mergeCell ref="I2:L2"/>
-    <mergeCell ref="M2:S2"/>
-    <mergeCell ref="A3:S3"/>
-    <mergeCell ref="A4:S4"/>
-    <mergeCell ref="A6:S6"/>
+    <mergeCell ref="M2:Q2"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="A4:Q4"/>
+    <mergeCell ref="A6:Q6"/>
     <mergeCell ref="A7:L7"/>
-    <mergeCell ref="A8:S8"/>
+    <mergeCell ref="A8:Q8"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true" horizontalCentered="true"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;C&amp;P / &amp;N · LightOn</oddFooter>
+    <oddFooter>&amp;C&amp;P / &amp;N · OnLight</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(catálogo): remover filtros avançados, valor com 2 decimais e export XLS no padrão BM
- Remove painel «Filtros avançados da tabela» (HTML, CSS e lógica JS); mantém ordenação por coluna
- Exibe valor unitário com 2 casas decimais (R$ 100,00) na tabela, modal e gravação (admin/cliente)
- Corrige export XLSX: compatibilidade PhpSpreadsheet 2.x (setCellValue em vez de setCellValueByColumnAndRow)
- Novo includes/catalogo_export_xlsx.php com layout institucional dos boletins de medição (capa roxa, zebrado, filtros)
</commit_message>
<xml_diff>
--- a/assets/templates/boletim_medicao_modelo_1.xlsx
+++ b/assets/templates/boletim_medicao_modelo_1.xlsx
@@ -10,7 +10,7 @@
     <sheet name="MEDIÇÃO" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'MEDIÇÃO'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'MEDIÇÃO'!$6:$6</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
@@ -22,8 +22,10 @@
     <t>BOLETIM DE MEDIÇÃO  ·  Nº 202605</t>
   </si>
   <si>
-    <t>Medição
-Modelo de referência</t>
+    <t>Medição Modelo de referência — —</t>
+  </si>
+  <si>
+    <t>Medição Modelo de referência · Valor total R$ 0,00</t>
   </si>
   <si>
     <t>Prefeitura / tomador
@@ -34,9 +36,10 @@
 —</t>
   </si>
   <si>
-    <t>Período / emitido
+    <t>Referência / emissão
 Modelo de referência
-15/05/2026 19:57</t>
+Gerado em
+18/05/2026 21:44</t>
   </si>
   <si>
     <t>Manutenção da iluminação pública — medição  ·  OnLight</t>
@@ -88,9 +91,6 @@
   </si>
   <si>
     <t>VALOR TOTAL (R$)</t>
-  </si>
-  <si>
-    <t>Material Retirados/Incluído</t>
   </si>
   <si>
     <t>Nenhum lançamento «utilizado» no período (filtro pela data em chamado_itens.criado_em; defina período nos filtros da lista de chamados).</t>
@@ -110,7 +110,7 @@
     <numFmt numFmtId="164" formatCode="&quot;R$&quot; #,##0.00"/>
     <numFmt numFmtId="165" formatCode="#,##0.###"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -143,7 +143,16 @@
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
-      <sz val="10"/>
+      <sz val="13"/>
+      <color rgb="FF534AB7"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="9"/>
       <color rgb="FFFFFFFF"/>
       <name val="Aptos"/>
     </font>
@@ -183,7 +192,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -204,7 +213,24 @@
       <left style="thin">
         <color rgb="FFBFC3D9"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color rgb="FFC9C6F4"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFC3D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFC3D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC9C6F4"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC9C6F4"/>
+      </right>
       <top style="thin">
         <color rgb="FFBFC3D9"/>
       </top>
@@ -295,16 +321,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false" indent="1"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="3" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false" indent="1"/>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false" indent="1"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="3" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false" indent="1"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="3" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false" indent="1"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="4" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false" indent="1"/>
@@ -312,29 +341,32 @@
     <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="5" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false" indent="1"/>
     </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="6" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="6" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false" indent="1"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="2" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="2" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false" indent="1"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="164" fillId="3" borderId="8" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="165" fillId="3" borderId="8" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="true"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="9" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="true" indent="1"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="9" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="true"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="164" fillId="3" borderId="9" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" shrinkToFit="true"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="165" fillId="3" borderId="9" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="true"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
   </cellXfs>
@@ -637,29 +669,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="true" style="0"/>
     <col min="2" max="2" width="10" customWidth="true" style="0"/>
-    <col min="3" max="3" width="16" customWidth="true" style="0"/>
-    <col min="4" max="4" width="16" customWidth="true" style="0"/>
-    <col min="5" max="5" width="20" customWidth="true" style="0"/>
-    <col min="6" max="6" width="18" customWidth="true" style="0"/>
+    <col min="3" max="3" width="18" customWidth="true" style="0"/>
+    <col min="4" max="4" width="18" customWidth="true" style="0"/>
+    <col min="5" max="5" width="22" customWidth="true" style="0"/>
+    <col min="6" max="6" width="20" customWidth="true" style="0"/>
     <col min="7" max="7" width="42" customWidth="true" style="0"/>
-    <col min="8" max="8" width="18" customWidth="true" style="0"/>
+    <col min="8" max="8" width="24" customWidth="true" style="0"/>
     <col min="9" max="9" width="22" customWidth="true" style="0"/>
-    <col min="10" max="10" width="18" customWidth="true" style="0"/>
-    <col min="11" max="11" width="16" customWidth="true" style="0"/>
-    <col min="12" max="12" width="48" customWidth="true" style="0"/>
+    <col min="10" max="10" width="22" customWidth="true" style="0"/>
+    <col min="11" max="11" width="14" customWidth="true" style="0"/>
+    <col min="12" max="12" width="44" customWidth="true" style="0"/>
     <col min="13" max="13" width="10" customWidth="true" style="0"/>
     <col min="14" max="14" width="8" customWidth="true" style="0"/>
-    <col min="15" max="15" width="18" customWidth="true" style="0"/>
-    <col min="16" max="16" width="18" customWidth="true" style="0"/>
-    <col min="17" max="17" width="28" customWidth="true" style="0"/>
+    <col min="15" max="15" width="20" customWidth="true" style="0"/>
+    <col min="16" max="16" width="20" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" customHeight="1" ht="54">
+    <row r="1" spans="1:16" customHeight="1" ht="40">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -678,207 +709,218 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="1:17" customHeight="1" ht="24">
+    <row r="2" spans="1:16" customHeight="1" ht="28">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="3" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+    </row>
+    <row r="3" spans="1:16" customHeight="1" ht="36">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="3" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="3" t="s">
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="7"/>
     </row>
-    <row r="3" spans="1:17" customHeight="1" ht="36">
-      <c r="A3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="6"/>
+    <row r="4" spans="1:16" customHeight="1" ht="32">
+      <c r="A4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
     </row>
-    <row r="4" spans="1:17" customHeight="1" ht="8">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7"/>
+    <row r="5" spans="1:16" customHeight="1" ht="8">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
     </row>
-    <row r="5" spans="1:17" customHeight="1" ht="40">
-      <c r="A5" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="8" t="s">
+    <row r="6" spans="1:16" customHeight="1" ht="38">
+      <c r="A6" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="B6" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="C6" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="D6" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="E6" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="F6" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="G6" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="H6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="I6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="J6" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="K6" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="8" t="s">
+      <c r="L6" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="N5" s="8" t="s">
+      <c r="M6" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="O5" s="8" t="s">
+      <c r="N6" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="P5" s="8" t="s">
+      <c r="O6" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="Q5" s="8" t="s">
+      <c r="P6" s="10" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
-      <c r="A6" s="9" t="s">
+    <row r="7" spans="1:16" customHeight="1" ht="28">
+      <c r="A7" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="9"/>
-    </row>
-    <row r="7" spans="1:17">
-      <c r="A7" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="13">
-        <v>0.0</v>
-      </c>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
       <c r="N7" s="11"/>
       <c r="O7" s="11"/>
-      <c r="P7" s="12">
+      <c r="P7" s="11"/>
+    </row>
+    <row r="8" spans="1:16" customHeight="1" ht="26">
+      <c r="A8" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
+      <c r="M8" s="15">
         <v>0.0</v>
       </c>
-      <c r="Q7" s="11"/>
+      <c r="N8" s="13"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="14">
+        <v>0.0</v>
+      </c>
     </row>
-    <row r="8" spans="1:17">
-      <c r="A8" s="14" t="s">
+    <row r="9" spans="1:16" customHeight="1" ht="28">
+      <c r="A9" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
-      <c r="P8" s="14"/>
-      <c r="Q8" s="14"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
     </row>
   </sheetData>
   <mergeCells>
-    <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="M2:Q2"/>
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A4:Q4"/>
-    <mergeCell ref="A6:Q6"/>
-    <mergeCell ref="A7:L7"/>
-    <mergeCell ref="A8:Q8"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="I3:L3"/>
+    <mergeCell ref="M3:P3"/>
+    <mergeCell ref="A4:P4"/>
+    <mergeCell ref="A5:P5"/>
+    <mergeCell ref="A7:P7"/>
+    <mergeCell ref="A8:L8"/>
+    <mergeCell ref="A9:P9"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true" horizontalCentered="true"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>

</xml_diff>